<commit_message>
fix(pivots): declare the table totals row so Excel opens it unrepaired; resumable captures
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KTccUzeFqqMqTthqgFm9H
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-pivots/table-totals-row.xlsx
+++ b/tests/fixtures/xlsx-pivots/table-totals-row.xlsx
@@ -63,11 +63,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:E7" headerRowCount="1" totalsRowCount="1">
   <autoFilter ref="A1:E6"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="Region"/>
+    <tableColumn id="1" name="Region" totalsRowLabel="Total"/>
     <tableColumn id="2" name="Product"/>
     <tableColumn id="3" name="Year"/>
-    <tableColumn id="4" name="Sales"/>
-    <tableColumn id="5" name="Units"/>
+    <tableColumn id="4" name="Sales" totalsRowFunction="sum"/>
+    <tableColumn id="5" name="Units" totalsRowFunction="sum"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -219,9 +219,11 @@
       <c r="B7"/>
       <c r="C7"/>
       <c r="D7">
+        <f>SUBTOTAL(109,Table1[Sales])</f>
         <v>21937.100000000002</v>
       </c>
       <c r="E7">
+        <f>SUBTOTAL(109,Table1[Units])</f>
         <v>279</v>
       </c>
     </row>

</xml_diff>